<commit_message>
automatic loops CryoGrid classes style
</commit_message>
<xml_diff>
--- a/CryoGrid/CryoGridCommunity_results/templates/no_spinup/no_spinup.xlsx
+++ b/CryoGrid/CryoGridCommunity_results/templates/no_spinup/no_spinup.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Utilisateurs\pozsgayv\Documents\CryoGrid_VP_Workflow\CryoGrid\CryoGridCommunity_results\templates\no_spinup\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E885FC94-9514-4415-B807-9D1C467EB17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF045F6F-8FAF-4CFD-A641-CA632FE7D3CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -609,9 +609,6 @@
     <t>include_Xice</t>
   </si>
   <si>
-    <t>TILE_1D_standard2</t>
-  </si>
-  <si>
     <t>init_steady_state_class</t>
   </si>
   <si>
@@ -733,6 +730,9 @@
   </si>
   <si>
     <t>D:\Utilisateurs\pozsgayv\Documents\CryoGrid_VP_Workflow\forcing\Forcing_Data\</t>
+  </si>
+  <si>
+    <t>TILE_1D</t>
   </si>
 </sst>
 </file>
@@ -1214,7 +1214,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -1247,7 +1247,7 @@
         <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>191</v>
+        <v>232</v>
       </c>
       <c r="D6" t="s">
         <v>24</v>
@@ -1271,7 +1271,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B8" t="s">
         <v>21</v>
@@ -1370,7 +1370,7 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="4"/>
@@ -1402,7 +1402,7 @@
     </row>
     <row r="28" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A28" s="9" t="s">
-        <v>191</v>
+        <v>232</v>
       </c>
       <c r="B28" s="9">
         <v>1</v>
@@ -1414,7 +1414,7 @@
         <v>8</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="31" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
@@ -1425,7 +1425,7 @@
         <v>100</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="32" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
@@ -1468,13 +1468,13 @@
         <v>21</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D36" s="9" t="s">
         <v>184</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F36" t="s">
         <v>24</v>
@@ -1533,7 +1533,7 @@
         <v>24</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="41" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
@@ -1561,7 +1561,7 @@
         <v>27</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="43" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
@@ -1586,7 +1586,7 @@
         <v>24</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="45" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
@@ -1605,37 +1605,37 @@
     </row>
     <row r="46" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="47" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="48" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B48">
         <v>-2</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="49" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B49">
         <v>0.5</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="50" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
@@ -1679,7 +1679,7 @@
         <v>32</v>
       </c>
       <c r="B56" s="17" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C56" s="15"/>
       <c r="D56" s="15"/>
@@ -1690,7 +1690,7 @@
         <v>33</v>
       </c>
       <c r="B57" s="18" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C57" s="15"/>
       <c r="D57" s="15"/>
@@ -1724,10 +1724,10 @@
         <v>21</v>
       </c>
       <c r="C59" s="17">
-        <v>2023</v>
+        <v>1958</v>
       </c>
       <c r="D59" s="17">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E59" s="17">
         <v>31</v>
@@ -1858,7 +1858,7 @@
     </row>
     <row r="76" spans="1:4" s="15" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A76" s="15" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B76" s="15">
         <v>1</v>
@@ -1916,7 +1916,7 @@
         <v>57</v>
       </c>
       <c r="B81" s="9" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D81" s="23" t="s">
         <v>58</v>
@@ -1942,13 +1942,13 @@
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A87" s="9" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B87">
         <v>1</v>
       </c>
       <c r="D87" s="8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.35">
@@ -1984,13 +1984,13 @@
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B90">
         <v>0</v>
       </c>
       <c r="D90" s="8" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H90" s="8"/>
     </row>
@@ -2002,7 +2002,7 @@
         <v>2844</v>
       </c>
       <c r="D91" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.35">
@@ -2013,7 +2013,7 @@
         <v>2790</v>
       </c>
       <c r="D92" s="8" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.35">
@@ -2065,7 +2065,7 @@
         <v>57</v>
       </c>
       <c r="B97" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D97" s="8" t="s">
         <v>58</v>
@@ -2175,7 +2175,7 @@
         <v>57</v>
       </c>
       <c r="B110" s="9" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="111" spans="1:14" outlineLevel="1" x14ac:dyDescent="0.35">
@@ -2424,7 +2424,7 @@
         <v>2</v>
       </c>
       <c r="D144" s="11" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="145" spans="1:10" x14ac:dyDescent="0.35">
@@ -2435,7 +2435,7 @@
         <v>1</v>
       </c>
       <c r="D145" s="11" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="147" spans="1:10" x14ac:dyDescent="0.35">
@@ -2544,7 +2544,7 @@
         <v>24</v>
       </c>
       <c r="G151" s="11" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="152" spans="1:10" x14ac:dyDescent="0.35">
@@ -2552,12 +2552,12 @@
         <v>6</v>
       </c>
       <c r="G152" s="11" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="153" spans="1:10" x14ac:dyDescent="0.35">
       <c r="G153" s="11" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="154" spans="1:10" s="15" customFormat="1" x14ac:dyDescent="0.35"/>
@@ -2623,7 +2623,7 @@
         <v>-2</v>
       </c>
       <c r="D161" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.35">
@@ -2735,7 +2735,7 @@
         <v>0.1</v>
       </c>
       <c r="D173" s="8" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.35">
@@ -2749,7 +2749,7 @@
         <v>0.1</v>
       </c>
       <c r="D174" s="8" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.35">
@@ -2763,7 +2763,7 @@
         <v>0.5</v>
       </c>
       <c r="D175" s="8" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.35">
@@ -2777,7 +2777,7 @@
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="D176" s="8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.35">
@@ -2990,7 +2990,7 @@
         <v>0</v>
       </c>
       <c r="D196" s="8" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.35">
@@ -3174,7 +3174,7 @@
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B215">
         <v>0</v>
@@ -3183,7 +3183,7 @@
         <v>0</v>
       </c>
       <c r="D215" s="8" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.35">
@@ -3249,7 +3249,7 @@
         <v>117</v>
       </c>
       <c r="C220" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D220" s="8" t="s">
         <v>93</v>

</xml_diff>

<commit_message>
New CryoGrid FORCING class: FORCING_seb_toElevation.m
</commit_message>
<xml_diff>
--- a/CryoGrid/CryoGridCommunity_results/templates/no_spinup/no_spinup.xlsx
+++ b/CryoGrid/CryoGridCommunity_results/templates/no_spinup/no_spinup.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Utilisateurs\pozsgayv\Documents\CryoGrid_VP_Workflow\CryoGrid\CryoGridCommunity_results\templates\no_spinup\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF045F6F-8FAF-4CFD-A641-CA632FE7D3CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BB733ED-414C-46D7-A483-8E26BA93A748}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="236">
   <si>
     <t>-------------------</t>
   </si>
@@ -729,10 +729,19 @@
     <t>snow_all</t>
   </si>
   <si>
-    <t>D:\Utilisateurs\pozsgayv\Documents\CryoGrid_VP_Workflow\forcing\Forcing_Data\</t>
-  </si>
-  <si>
     <t>TILE_1D</t>
+  </si>
+  <si>
+    <t>FORCING_seb_toElevation</t>
+  </si>
+  <si>
+    <t>..\..\forcing\Forcing_Data\</t>
+  </si>
+  <si>
+    <t>FORCING_SAFRAN_ALL</t>
+  </si>
+  <si>
+    <t>..\..\forcing\Forcing_Data\meteo\CryoGrid_ready_new\</t>
   </si>
 </sst>
 </file>
@@ -829,13 +838,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
@@ -856,9 +862,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1219,7 +1222,7 @@
       <c r="B3">
         <v>1</v>
       </c>
-      <c r="G3" s="15"/>
+      <c r="G3" s="14"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -1228,7 +1231,7 @@
       <c r="B4" t="s">
         <v>180</v>
       </c>
-      <c r="G4" s="15"/>
+      <c r="G4" s="14"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
@@ -1237,7 +1240,7 @@
       <c r="B5">
         <v>1</v>
       </c>
-      <c r="G5" s="15"/>
+      <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
@@ -1247,12 +1250,12 @@
         <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D6" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="15"/>
+      <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
@@ -1267,7 +1270,7 @@
       <c r="D7" t="s">
         <v>24</v>
       </c>
-      <c r="G7" s="15"/>
+      <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
@@ -1282,13 +1285,13 @@
       <c r="D8" t="s">
         <v>24</v>
       </c>
-      <c r="G8" s="15"/>
+      <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>6</v>
       </c>
-      <c r="G9" s="15"/>
+      <c r="G9" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
@@ -1315,125 +1318,131 @@
       <c r="A15" t="s">
         <v>156</v>
       </c>
-      <c r="B15" s="5">
-        <v>45.3</v>
+      <c r="B15" s="4">
+        <v>45.897941600000003</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>157</v>
       </c>
-      <c r="B16" s="5">
-        <v>6.6</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B16" s="4">
+        <v>6.8235998000000002</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>158</v>
       </c>
-      <c r="B17" s="5">
+      <c r="B17" s="4">
         <v>2840</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" s="12" t="s">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" s="11" t="s">
         <v>174</v>
       </c>
-      <c r="B18" s="13">
+      <c r="B18" s="12">
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" s="12" t="s">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" s="11" t="s">
         <v>175</v>
       </c>
-      <c r="B19" s="13">
+      <c r="B19" s="12">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A20" s="12" t="s">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" s="11" t="s">
         <v>183</v>
       </c>
-      <c r="B20" s="14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B20" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>159</v>
       </c>
       <c r="B21">
         <v>1</v>
       </c>
-      <c r="C21" s="7"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C21" s="6"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>205</v>
       </c>
-      <c r="C22" s="7"/>
-      <c r="D22" s="4"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C22" s="6"/>
+      <c r="D22" s="3"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>6</v>
       </c>
-      <c r="D23" s="4"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="D24" s="4"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="D25" s="4"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D23" s="3"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="D24" s="3"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="D25" s="3"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="9" t="s">
+    <row r="27" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="8" t="s">
         <v>7</v>
       </c>
       <c r="B27" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="9" t="s">
-        <v>232</v>
-      </c>
-      <c r="B28" s="9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35"/>
-    <row r="30" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="B28" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35"/>
+    <row r="30" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>8</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="B30" s="8" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="31" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>9</v>
       </c>
       <c r="B31">
         <v>100</v>
       </c>
-      <c r="C31" s="8" t="s">
+      <c r="C31" s="7" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="32" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" t="s">
+        <v>232</v>
+      </c>
+      <c r="E32" t="s">
         <v>177</v>
+      </c>
+      <c r="F32" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="33" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
@@ -1467,13 +1476,13 @@
       <c r="B36" t="s">
         <v>21</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="C36" s="8" t="s">
         <v>221</v>
       </c>
-      <c r="D36" s="9" t="s">
+      <c r="D36" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="E36" s="9" t="s">
+      <c r="E36" s="8" t="s">
         <v>226</v>
       </c>
       <c r="F36" t="s">
@@ -1487,13 +1496,13 @@
       <c r="B37" t="s">
         <v>21</v>
       </c>
-      <c r="C37" s="9">
-        <v>1</v>
-      </c>
-      <c r="D37" s="9">
-        <v>1</v>
-      </c>
-      <c r="E37" s="9">
+      <c r="C37" s="8">
+        <v>1</v>
+      </c>
+      <c r="D37" s="8">
+        <v>1</v>
+      </c>
+      <c r="E37" s="8">
         <v>1</v>
       </c>
       <c r="F37" t="s">
@@ -1532,7 +1541,7 @@
       <c r="E40" t="s">
         <v>24</v>
       </c>
-      <c r="F40" s="8" t="s">
+      <c r="F40" s="7" t="s">
         <v>207</v>
       </c>
     </row>
@@ -1560,7 +1569,7 @@
       <c r="B42" t="s">
         <v>27</v>
       </c>
-      <c r="C42" s="8" t="s">
+      <c r="C42" s="7" t="s">
         <v>208</v>
       </c>
     </row>
@@ -1585,7 +1594,7 @@
       <c r="D44" t="s">
         <v>24</v>
       </c>
-      <c r="E44" s="8" t="s">
+      <c r="E44" s="7" t="s">
         <v>209</v>
       </c>
     </row>
@@ -1607,7 +1616,7 @@
       <c r="A46" t="s">
         <v>191</v>
       </c>
-      <c r="C46" s="8" t="s">
+      <c r="C46" s="7" t="s">
         <v>210</v>
       </c>
     </row>
@@ -1623,7 +1632,7 @@
       <c r="B48">
         <v>-2</v>
       </c>
-      <c r="C48" s="8" t="s">
+      <c r="C48" s="7" t="s">
         <v>211</v>
       </c>
     </row>
@@ -1634,7 +1643,7 @@
       <c r="B49">
         <v>0.5</v>
       </c>
-      <c r="C49" s="8" t="s">
+      <c r="C49" s="7" t="s">
         <v>212</v>
       </c>
     </row>
@@ -1645,7 +1654,7 @@
     </row>
     <row r="51" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35"/>
     <row r="52" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="D52" s="4"/>
+      <c r="D52" s="3"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
@@ -1653,63 +1662,77 @@
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A54" s="15" t="s">
+      <c r="A54" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="B54" s="15" t="s">
+      <c r="B54" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C54" s="15"/>
-      <c r="D54" s="15"/>
-      <c r="E54" s="15"/>
+      <c r="C54" s="14"/>
+      <c r="D54" s="14"/>
+      <c r="E54" s="14"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A55" s="16" t="s">
+      <c r="A55" t="s">
+        <v>232</v>
+      </c>
+      <c r="B55" s="16">
+        <v>1</v>
+      </c>
+      <c r="C55" s="14"/>
+      <c r="E55" t="s">
+        <v>232</v>
+      </c>
+      <c r="F55" t="s">
         <v>177</v>
       </c>
-      <c r="B55" s="18">
-        <v>1</v>
-      </c>
-      <c r="C55" s="15"/>
-      <c r="D55" s="15"/>
-      <c r="E55" s="15"/>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A56" s="17" t="s">
+      <c r="A56" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="B56" s="17" t="s">
+      <c r="B56" s="15" t="s">
+        <v>234</v>
+      </c>
+      <c r="C56" s="14"/>
+      <c r="D56" s="14"/>
+      <c r="E56" s="15" t="s">
+        <v>234</v>
+      </c>
+      <c r="F56" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="C56" s="15"/>
-      <c r="D56" s="15"/>
-      <c r="E56" s="15"/>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A57" s="15" t="s">
+      <c r="A57" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B57" s="18" t="s">
-        <v>231</v>
-      </c>
-      <c r="C57" s="15"/>
-      <c r="D57" s="15"/>
-      <c r="E57" s="15"/>
+      <c r="B57" s="16" t="s">
+        <v>235</v>
+      </c>
+      <c r="C57" s="14"/>
+      <c r="D57" s="14"/>
+      <c r="E57" s="16" t="s">
+        <v>235</v>
+      </c>
+      <c r="F57" s="16" t="s">
+        <v>233</v>
+      </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A58" s="15" t="s">
+      <c r="A58" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="B58" s="15" t="s">
+      <c r="B58" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C58" s="17">
+      <c r="C58" s="15">
         <v>1958</v>
       </c>
-      <c r="D58" s="17">
+      <c r="D58" s="15">
         <v>9</v>
       </c>
-      <c r="E58" s="17">
+      <c r="E58" s="15">
         <v>1</v>
       </c>
       <c r="F58" t="s">
@@ -1717,83 +1740,82 @@
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A59" s="15" t="s">
+      <c r="A59" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="B59" s="15" t="s">
+      <c r="B59" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C59" s="17">
+      <c r="C59" s="15">
         <v>1958</v>
       </c>
-      <c r="D59" s="17">
+      <c r="D59" s="15">
         <v>9</v>
       </c>
-      <c r="E59" s="17">
-        <v>31</v>
+      <c r="E59" s="15">
+        <v>10</v>
       </c>
       <c r="F59" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A60" s="15" t="s">
+      <c r="A60" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="B60" s="15">
-        <v>1</v>
-      </c>
-      <c r="C60" s="15"/>
-      <c r="D60" s="15"/>
-      <c r="E60" s="15"/>
+      <c r="B60" s="14">
+        <v>1</v>
+      </c>
+      <c r="C60" s="14"/>
+      <c r="D60" s="14"/>
+      <c r="E60" s="14"/>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A61" s="19" t="s">
+      <c r="A61" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="B61" s="20">
-        <v>1</v>
-      </c>
-      <c r="C61" s="15"/>
-      <c r="D61" s="15"/>
-      <c r="E61" s="15"/>
+      <c r="B61" s="18">
+        <v>1</v>
+      </c>
+      <c r="C61" s="14"/>
+      <c r="D61" s="14"/>
+      <c r="E61" s="14"/>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A62" s="15" t="s">
+      <c r="A62" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="B62" s="15">
-        <v>0</v>
-      </c>
-      <c r="C62" s="15"/>
-      <c r="D62" s="15"/>
-      <c r="E62" s="15"/>
+      <c r="B62" s="14">
+        <v>0.5</v>
+      </c>
+      <c r="C62" s="14"/>
+      <c r="D62" s="14"/>
+      <c r="E62" s="14"/>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A63" s="15" t="s">
+      <c r="A63" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="B63" s="15">
+      <c r="B63" s="14">
         <v>2</v>
       </c>
-      <c r="C63" s="15"/>
-      <c r="D63" s="15"/>
-      <c r="E63" s="15"/>
+      <c r="C63" s="14"/>
+      <c r="D63" s="14"/>
+      <c r="E63" s="14"/>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A64" s="15" t="s">
+      <c r="A64" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="B64" s="15" t="s">
+      <c r="B64" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C64" s="18" t="s">
+      <c r="C64" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="D64" s="16" t="s">
         <v>176</v>
       </c>
-      <c r="D64" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="E64" s="15"/>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
@@ -1802,11 +1824,11 @@
       <c r="B65" t="s">
         <v>21</v>
       </c>
-      <c r="C65">
-        <v>1</v>
-      </c>
-      <c r="D65" t="s">
+      <c r="C65" t="s">
         <v>24</v>
+      </c>
+      <c r="D65">
+        <v>1</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
@@ -1815,18 +1837,18 @@
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A68" s="9" t="s">
+      <c r="A68" s="8" t="s">
         <v>181</v>
       </c>
-      <c r="B68" s="9" t="s">
+      <c r="B68" s="8" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A69" s="9" t="s">
+      <c r="A69" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="B69" s="9">
+      <c r="B69" s="8">
         <v>1</v>
       </c>
     </row>
@@ -1843,87 +1865,87 @@
         <v>6</v>
       </c>
     </row>
-    <row r="74" spans="1:4" s="15" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A74" s="15" t="s">
+    <row r="74" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A74" s="14" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:4" s="15" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A75" s="15" t="s">
+    <row r="75" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A75" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="B75" s="15" t="s">
+      <c r="B75" s="14" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="76" spans="1:4" s="15" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A76" s="15" t="s">
+    <row r="76" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A76" s="14" t="s">
         <v>226</v>
       </c>
-      <c r="B76" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" s="15" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C77" s="15" t="s">
+      <c r="B76" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="C77" s="14" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="78" spans="1:4" s="15" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A78" s="15" t="s">
+    <row r="78" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A78" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="B78" s="15">
+      <c r="B78" s="14">
         <v>0.25</v>
       </c>
-      <c r="C78" s="15">
+      <c r="C78" s="14">
         <v>0.25</v>
       </c>
-      <c r="D78" s="23" t="s">
+      <c r="D78" s="21" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="79" spans="1:4" s="15" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A79" s="15" t="s">
+    <row r="79" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A79" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="B79" s="15" t="s">
+      <c r="B79" s="14" t="s">
         <v>173</v>
       </c>
-      <c r="C79" s="15" t="s">
+      <c r="C79" s="14" t="s">
         <v>173</v>
       </c>
-      <c r="D79" s="23" t="s">
+      <c r="D79" s="21" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="80" spans="1:4" s="15" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A80" s="15" t="s">
+    <row r="80" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A80" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="B80" s="15">
+      <c r="B80" s="14">
         <v>5</v>
       </c>
-      <c r="C80" s="15">
-        <v>1</v>
-      </c>
-      <c r="D80" s="23" t="s">
+      <c r="C80" s="14">
+        <v>1</v>
+      </c>
+      <c r="D80" s="21" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="81" spans="1:8" s="15" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A81" s="9" t="s">
+    <row r="81" spans="1:8" s="14" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A81" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="B81" s="9" t="s">
+      <c r="B81" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="D81" s="23" t="s">
+      <c r="D81" s="21" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="82" spans="1:8" s="15" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A82" s="15" t="s">
+    <row r="82" spans="1:8" s="14" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A82" s="14" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1941,13 +1963,13 @@
       </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A87" s="9" t="s">
+      <c r="A87" s="8" t="s">
         <v>221</v>
       </c>
       <c r="B87">
         <v>1</v>
       </c>
-      <c r="D87" s="8" t="s">
+      <c r="D87" s="7" t="s">
         <v>227</v>
       </c>
     </row>
@@ -1978,7 +2000,7 @@
       <c r="G89" t="s">
         <v>24</v>
       </c>
-      <c r="H89" s="8" t="s">
+      <c r="H89" s="7" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1989,10 +2011,10 @@
       <c r="B90">
         <v>0</v>
       </c>
-      <c r="D90" s="8" t="s">
+      <c r="D90" s="7" t="s">
         <v>223</v>
       </c>
-      <c r="H90" s="8"/>
+      <c r="H90" s="7"/>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
@@ -2001,7 +2023,7 @@
       <c r="B91">
         <v>2844</v>
       </c>
-      <c r="D91" s="8" t="s">
+      <c r="D91" s="7" t="s">
         <v>224</v>
       </c>
     </row>
@@ -2012,7 +2034,7 @@
       <c r="B92">
         <v>2790</v>
       </c>
-      <c r="D92" s="8" t="s">
+      <c r="D92" s="7" t="s">
         <v>225</v>
       </c>
     </row>
@@ -2023,7 +2045,7 @@
       <c r="B93">
         <v>0.1</v>
       </c>
-      <c r="D93" s="8" t="s">
+      <c r="D93" s="7" t="s">
         <v>50</v>
       </c>
     </row>
@@ -2034,7 +2056,7 @@
       <c r="B94">
         <v>0.25</v>
       </c>
-      <c r="D94" s="8" t="s">
+      <c r="D94" s="7" t="s">
         <v>52</v>
       </c>
     </row>
@@ -2045,7 +2067,7 @@
       <c r="B95" t="s">
         <v>173</v>
       </c>
-      <c r="D95" s="8" t="s">
+      <c r="D95" s="7" t="s">
         <v>54</v>
       </c>
     </row>
@@ -2056,18 +2078,18 @@
       <c r="B96">
         <v>5</v>
       </c>
-      <c r="D96" s="8" t="s">
+      <c r="D96" s="7" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="97" spans="1:14" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A97" s="5" t="s">
+      <c r="A97" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B97" s="5" t="s">
+      <c r="B97" s="4" t="s">
         <v>229</v>
       </c>
-      <c r="D97" s="8" t="s">
+      <c r="D97" s="7" t="s">
         <v>58</v>
       </c>
     </row>
@@ -2077,18 +2099,18 @@
       </c>
     </row>
     <row r="101" spans="1:14" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A101" s="9" t="s">
+      <c r="A101" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B101" s="9" t="s">
+      <c r="B101" s="8" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="102" spans="1:14" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A102" s="9" t="s">
+      <c r="A102" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="B102" s="9">
+      <c r="B102" s="8">
         <v>1</v>
       </c>
     </row>
@@ -2165,16 +2187,16 @@
       <c r="B109">
         <v>5</v>
       </c>
-      <c r="I109" s="10"/>
-      <c r="J109" s="10"/>
-      <c r="K109" s="10"/>
-      <c r="N109" s="10"/>
+      <c r="I109" s="9"/>
+      <c r="J109" s="9"/>
+      <c r="K109" s="9"/>
+      <c r="N109" s="9"/>
     </row>
     <row r="110" spans="1:14" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A110" s="9" t="s">
+      <c r="A110" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="B110" s="9" t="s">
+      <c r="B110" s="8" t="s">
         <v>230</v>
       </c>
     </row>
@@ -2328,7 +2350,7 @@
       <c r="E132" t="s">
         <v>24</v>
       </c>
-      <c r="F132" s="8" t="s">
+      <c r="F132" s="7" t="s">
         <v>70</v>
       </c>
     </row>
@@ -2353,7 +2375,7 @@
       <c r="D134">
         <v>1</v>
       </c>
-      <c r="F134" s="8" t="s">
+      <c r="F134" s="7" t="s">
         <v>169</v>
       </c>
     </row>
@@ -2369,7 +2391,7 @@
       <c r="B136" t="s">
         <v>160</v>
       </c>
-      <c r="D136" s="8" t="s">
+      <c r="D136" s="7" t="s">
         <v>72</v>
       </c>
     </row>
@@ -2391,7 +2413,7 @@
       <c r="C138" t="s">
         <v>24</v>
       </c>
-      <c r="D138" s="8" t="s">
+      <c r="D138" s="7" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2423,7 +2445,7 @@
       <c r="B144" t="s">
         <v>2</v>
       </c>
-      <c r="D144" s="11" t="s">
+      <c r="D144" s="10" t="s">
         <v>200</v>
       </c>
     </row>
@@ -2434,7 +2456,7 @@
       <c r="B145">
         <v>1</v>
       </c>
-      <c r="D145" s="11" t="s">
+      <c r="D145" s="10" t="s">
         <v>201</v>
       </c>
     </row>
@@ -2466,7 +2488,7 @@
       <c r="I147" t="s">
         <v>24</v>
       </c>
-      <c r="J147" s="8" t="s">
+      <c r="J147" s="7" t="s">
         <v>178</v>
       </c>
     </row>
@@ -2489,7 +2511,7 @@
       <c r="G148">
         <v>0.2</v>
       </c>
-      <c r="H148" s="22">
+      <c r="H148" s="20">
         <v>9.9999999999999995E-7</v>
       </c>
     </row>
@@ -2512,7 +2534,7 @@
       <c r="G149">
         <v>0.2</v>
       </c>
-      <c r="H149" s="22">
+      <c r="H149" s="20">
         <v>9.9999999999999995E-7</v>
       </c>
     </row>
@@ -2535,7 +2557,7 @@
       <c r="G150">
         <v>0.03</v>
       </c>
-      <c r="H150" s="22">
+      <c r="H150" s="20">
         <v>9.9999999999999995E-7</v>
       </c>
     </row>
@@ -2543,7 +2565,7 @@
       <c r="B151" t="s">
         <v>24</v>
       </c>
-      <c r="G151" s="11" t="s">
+      <c r="G151" s="10" t="s">
         <v>202</v>
       </c>
     </row>
@@ -2551,54 +2573,54 @@
       <c r="A152" t="s">
         <v>6</v>
       </c>
-      <c r="G152" s="11" t="s">
+      <c r="G152" s="10" t="s">
         <v>203</v>
       </c>
     </row>
     <row r="153" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="G153" s="11" t="s">
+      <c r="G153" s="10" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="154" spans="1:10" s="15" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="154" spans="1:10" s="14" customFormat="1" x14ac:dyDescent="0.35"/>
     <row r="155" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A155" s="15" t="s">
+      <c r="A155" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B155" s="15"/>
-      <c r="C155" s="15"/>
+      <c r="B155" s="14"/>
+      <c r="C155" s="14"/>
     </row>
     <row r="156" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A156" s="15" t="s">
+      <c r="A156" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="B156" s="15" t="s">
+      <c r="B156" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C156" s="15"/>
+      <c r="C156" s="14"/>
     </row>
     <row r="157" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A157" s="15" t="s">
+      <c r="A157" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="B157" s="15">
-        <v>1</v>
-      </c>
-      <c r="C157" s="15"/>
+      <c r="B157" s="14">
+        <v>1</v>
+      </c>
+      <c r="C157" s="14"/>
     </row>
     <row r="158" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A158" s="15"/>
-      <c r="B158" s="15"/>
-      <c r="C158" s="15"/>
+      <c r="A158" s="14"/>
+      <c r="B158" s="14"/>
+      <c r="C158" s="14"/>
     </row>
     <row r="159" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A159" s="15" t="s">
+      <c r="A159" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="B159" s="15" t="s">
+      <c r="B159" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="C159" s="17" t="s">
+      <c r="C159" s="15" t="s">
         <v>42</v>
       </c>
       <c r="D159" t="s">
@@ -2606,20 +2628,20 @@
       </c>
     </row>
     <row r="160" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A160" s="15"/>
-      <c r="B160" s="15">
+      <c r="A160" s="14"/>
+      <c r="B160" s="14">
         <v>0</v>
       </c>
-      <c r="C160" s="17">
+      <c r="C160" s="15">
         <v>-2</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A161" s="15"/>
-      <c r="B161" s="17">
+      <c r="A161" s="14"/>
+      <c r="B161" s="15">
         <v>100</v>
       </c>
-      <c r="C161" s="17">
+      <c r="C161" s="15">
         <v>-2</v>
       </c>
       <c r="D161" t="s">
@@ -2627,170 +2649,170 @@
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A162" s="15"/>
-      <c r="B162" s="15" t="s">
+      <c r="A162" s="14"/>
+      <c r="B162" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="C162" s="21"/>
+      <c r="C162" s="19"/>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A163" s="15" t="s">
+      <c r="A163" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="B163" s="15"/>
-      <c r="C163" s="15"/>
+      <c r="B163" s="14"/>
+      <c r="C163" s="14"/>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A164" s="15"/>
-      <c r="B164" s="15"/>
-      <c r="C164" s="15"/>
+      <c r="A164" s="14"/>
+      <c r="B164" s="14"/>
+      <c r="C164" s="14"/>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A165" s="15"/>
-      <c r="B165" s="15"/>
-      <c r="C165" s="15"/>
+      <c r="A165" s="14"/>
+      <c r="B165" s="14"/>
+      <c r="C165" s="14"/>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A166" s="15" t="s">
+      <c r="A166" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B166" s="15"/>
-      <c r="C166" s="15"/>
+      <c r="B166" s="14"/>
+      <c r="C166" s="14"/>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A167" s="15" t="s">
+      <c r="A167" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="B167" s="15" t="s">
+      <c r="B167" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C167" s="15"/>
+      <c r="C167" s="14"/>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A168" s="15" t="s">
+      <c r="A168" s="14" t="s">
         <v>161</v>
       </c>
-      <c r="B168" s="15">
-        <v>1</v>
-      </c>
-      <c r="C168" s="15"/>
+      <c r="B168" s="14">
+        <v>1</v>
+      </c>
+      <c r="C168" s="14"/>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A169" s="15"/>
-      <c r="B169" s="15"/>
-      <c r="C169" s="15" t="s">
+      <c r="A169" s="14"/>
+      <c r="B169" s="14"/>
+      <c r="C169" s="14" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A170" s="17" t="s">
+      <c r="A170" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="B170" s="17">
+      <c r="B170" s="15">
         <v>0.25</v>
       </c>
-      <c r="C170" s="15">
+      <c r="C170" s="14">
         <v>0.2</v>
       </c>
-      <c r="D170" s="8" t="s">
+      <c r="D170" s="7" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A171" s="15" t="s">
+      <c r="A171" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="B171" s="15">
+      <c r="B171" s="14">
         <v>0.99</v>
       </c>
-      <c r="C171" s="15">
+      <c r="C171" s="14">
         <v>0.99</v>
       </c>
-      <c r="D171" s="8" t="s">
+      <c r="D171" s="7" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A172" s="18" t="s">
+      <c r="A172" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="B172" s="18">
+      <c r="B172" s="16">
         <v>0.27</v>
       </c>
-      <c r="C172" s="15">
+      <c r="C172" s="14">
         <v>0.01</v>
       </c>
-      <c r="D172" s="8" t="s">
+      <c r="D172" s="7" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A173" s="15" t="s">
+      <c r="A173" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="B173" s="15">
+      <c r="B173" s="14">
         <v>0.1</v>
       </c>
-      <c r="C173" s="15">
+      <c r="C173" s="14">
         <v>0.1</v>
       </c>
-      <c r="D173" s="8" t="s">
+      <c r="D173" s="7" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A174" s="15" t="s">
+      <c r="A174" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="B174" s="15">
+      <c r="B174" s="14">
         <v>0.1</v>
       </c>
-      <c r="C174" s="15">
+      <c r="C174" s="14">
         <v>0.1</v>
       </c>
-      <c r="D174" s="8" t="s">
+      <c r="D174" s="7" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A175" s="15" t="s">
+      <c r="A175" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="B175" s="15">
+      <c r="B175" s="14">
         <v>0.5</v>
       </c>
-      <c r="C175" s="15">
+      <c r="C175" s="14">
         <v>0.5</v>
       </c>
-      <c r="D175" s="8" t="s">
+      <c r="D175" s="7" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A176" s="15" t="s">
+      <c r="A176" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="B176" s="15">
+      <c r="B176" s="14">
         <v>1.0000000000000001E-5</v>
       </c>
-      <c r="C176" s="15">
+      <c r="C176" s="14">
         <v>1.0000000000000001E-5</v>
       </c>
-      <c r="D176" s="8" t="s">
+      <c r="D176" s="7" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A177" s="15" t="s">
+      <c r="A177" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="B177" s="15" t="s">
+      <c r="B177" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="C177" s="15" t="s">
+      <c r="C177" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="D177" s="8" t="s">
+      <c r="D177" s="7" t="s">
         <v>93</v>
       </c>
     </row>
@@ -2804,7 +2826,7 @@
       <c r="C178">
         <v>3600</v>
       </c>
-      <c r="D178" s="8" t="s">
+      <c r="D178" s="7" t="s">
         <v>95</v>
       </c>
     </row>
@@ -2818,7 +2840,7 @@
       <c r="C179">
         <v>50000</v>
       </c>
-      <c r="D179" s="8" t="s">
+      <c r="D179" s="7" t="s">
         <v>97</v>
       </c>
     </row>
@@ -2832,7 +2854,7 @@
       <c r="C180">
         <v>1000</v>
       </c>
-      <c r="D180" s="8" t="s">
+      <c r="D180" s="7" t="s">
         <v>153</v>
       </c>
     </row>
@@ -2846,7 +2868,7 @@
       <c r="C181">
         <v>1000</v>
       </c>
-      <c r="D181" s="8" t="s">
+      <c r="D181" s="7" t="s">
         <v>155</v>
       </c>
     </row>
@@ -2860,7 +2882,7 @@
       <c r="C182">
         <v>-50</v>
       </c>
-      <c r="D182" s="8" t="s">
+      <c r="D182" s="7" t="s">
         <v>145</v>
       </c>
     </row>
@@ -2874,7 +2896,7 @@
       <c r="C183">
         <v>0.05</v>
       </c>
-      <c r="D183" s="8" t="s">
+      <c r="D183" s="7" t="s">
         <v>147</v>
       </c>
     </row>
@@ -2888,7 +2910,7 @@
       <c r="C184">
         <v>0.97</v>
       </c>
-      <c r="D184" s="8" t="s">
+      <c r="D184" s="7" t="s">
         <v>149</v>
       </c>
     </row>
@@ -2902,7 +2924,7 @@
       <c r="C185">
         <v>0.03</v>
       </c>
-      <c r="D185" s="8" t="s">
+      <c r="D185" s="7" t="s">
         <v>151</v>
       </c>
     </row>
@@ -2941,13 +2963,13 @@
       <c r="A193" t="s">
         <v>84</v>
       </c>
-      <c r="B193" s="9">
+      <c r="B193" s="8">
         <v>0.25</v>
       </c>
       <c r="C193">
         <v>0.2</v>
       </c>
-      <c r="D193" s="8" t="s">
+      <c r="D193" s="7" t="s">
         <v>85</v>
       </c>
     </row>
@@ -2961,7 +2983,7 @@
       <c r="C194">
         <v>0.99</v>
       </c>
-      <c r="D194" s="8" t="s">
+      <c r="D194" s="7" t="s">
         <v>87</v>
       </c>
     </row>
@@ -2969,13 +2991,13 @@
       <c r="A195" t="s">
         <v>88</v>
       </c>
-      <c r="B195" s="18">
+      <c r="B195" s="16">
         <v>0.27</v>
       </c>
       <c r="C195">
         <v>0.01</v>
       </c>
-      <c r="D195" s="8" t="s">
+      <c r="D195" s="7" t="s">
         <v>89</v>
       </c>
     </row>
@@ -2989,7 +3011,7 @@
       <c r="C196">
         <v>0</v>
       </c>
-      <c r="D196" s="8" t="s">
+      <c r="D196" s="7" t="s">
         <v>217</v>
       </c>
     </row>
@@ -3003,7 +3025,7 @@
       <c r="C197" t="s">
         <v>92</v>
       </c>
-      <c r="D197" s="8" t="s">
+      <c r="D197" s="7" t="s">
         <v>93</v>
       </c>
     </row>
@@ -3017,7 +3039,7 @@
       <c r="C198">
         <v>3600</v>
       </c>
-      <c r="D198" s="8" t="s">
+      <c r="D198" s="7" t="s">
         <v>95</v>
       </c>
     </row>
@@ -3031,7 +3053,7 @@
       <c r="C199">
         <v>50000</v>
       </c>
-      <c r="D199" s="8" t="s">
+      <c r="D199" s="7" t="s">
         <v>97</v>
       </c>
     </row>
@@ -3076,7 +3098,7 @@
       <c r="C207">
         <v>0.99</v>
       </c>
-      <c r="D207" s="8" t="s">
+      <c r="D207" s="7" t="s">
         <v>87</v>
       </c>
     </row>
@@ -3090,7 +3112,7 @@
       <c r="C208">
         <v>0.01</v>
       </c>
-      <c r="D208" s="8" t="s">
+      <c r="D208" s="7" t="s">
         <v>89</v>
       </c>
     </row>
@@ -3104,7 +3126,7 @@
       <c r="C209">
         <v>0.71</v>
       </c>
-      <c r="D209" s="8" t="s">
+      <c r="D209" s="7" t="s">
         <v>100</v>
       </c>
     </row>
@@ -3118,7 +3140,7 @@
       <c r="C210">
         <v>0.21</v>
       </c>
-      <c r="D210" s="8" t="s">
+      <c r="D210" s="7" t="s">
         <v>102</v>
       </c>
     </row>
@@ -3126,7 +3148,7 @@
       <c r="A211" t="s">
         <v>103</v>
       </c>
-      <c r="D211" s="8" t="s">
+      <c r="D211" s="7" t="s">
         <v>104</v>
       </c>
     </row>
@@ -3140,7 +3162,7 @@
       <c r="C212">
         <v>0.05</v>
       </c>
-      <c r="D212" s="8" t="s">
+      <c r="D212" s="7" t="s">
         <v>105</v>
       </c>
     </row>
@@ -3154,7 +3176,7 @@
       <c r="C213">
         <v>1E-4</v>
       </c>
-      <c r="D213" s="8" t="s">
+      <c r="D213" s="7" t="s">
         <v>106</v>
       </c>
     </row>
@@ -3168,7 +3190,7 @@
       <c r="C214">
         <v>0.02</v>
       </c>
-      <c r="D214" s="8" t="s">
+      <c r="D214" s="7" t="s">
         <v>108</v>
       </c>
     </row>
@@ -3182,7 +3204,7 @@
       <c r="C215">
         <v>0</v>
       </c>
-      <c r="D215" s="8" t="s">
+      <c r="D215" s="7" t="s">
         <v>219</v>
       </c>
     </row>
@@ -3197,7 +3219,7 @@
       <c r="C216">
         <v>48</v>
       </c>
-      <c r="D216" s="8" t="s">
+      <c r="D216" s="7" t="s">
         <v>110</v>
       </c>
     </row>
@@ -3211,7 +3233,7 @@
       <c r="C217">
         <v>350</v>
       </c>
-      <c r="D217" s="8" t="s">
+      <c r="D217" s="7" t="s">
         <v>112</v>
       </c>
     </row>
@@ -3225,7 +3247,7 @@
       <c r="C218">
         <v>26</v>
       </c>
-      <c r="D218" s="8" t="s">
+      <c r="D218" s="7" t="s">
         <v>114</v>
       </c>
     </row>
@@ -3237,7 +3259,7 @@
         <f>0.06/60</f>
         <v>1E-3</v>
       </c>
-      <c r="D219" s="8" t="s">
+      <c r="D219" s="7" t="s">
         <v>116</v>
       </c>
     </row>
@@ -3251,7 +3273,7 @@
       <c r="C220" t="s">
         <v>220</v>
       </c>
-      <c r="D220" s="8" t="s">
+      <c r="D220" s="7" t="s">
         <v>93</v>
       </c>
     </row>
@@ -3265,7 +3287,7 @@
       <c r="C221">
         <v>3600</v>
       </c>
-      <c r="D221" s="8" t="s">
+      <c r="D221" s="7" t="s">
         <v>95</v>
       </c>
     </row>
@@ -3279,7 +3301,7 @@
       <c r="C222">
         <v>50000</v>
       </c>
-      <c r="D222" s="8" t="s">
+      <c r="D222" s="7" t="s">
         <v>97</v>
       </c>
     </row>
@@ -3287,7 +3309,7 @@
       <c r="A223" t="s">
         <v>137</v>
       </c>
-      <c r="D223" s="8"/>
+      <c r="D223" s="7"/>
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
@@ -3295,10 +3317,10 @@
       </c>
     </row>
     <row r="225" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="D225" s="8"/>
+      <c r="D225" s="7"/>
     </row>
     <row r="226" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="D226" s="8"/>
+      <c r="D226" s="7"/>
     </row>
     <row r="227" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
@@ -3320,7 +3342,7 @@
       <c r="B229">
         <v>1</v>
       </c>
-      <c r="D229" s="8" t="s">
+      <c r="D229" s="7" t="s">
         <v>170</v>
       </c>
     </row>
@@ -3339,7 +3361,7 @@
       <c r="C231">
         <v>0.25</v>
       </c>
-      <c r="D231" s="8" t="s">
+      <c r="D231" s="7" t="s">
         <v>120</v>
       </c>
     </row>
@@ -3349,10 +3371,10 @@
       </c>
     </row>
     <row r="233" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="D233" s="8"/>
+      <c r="D233" s="7"/>
     </row>
     <row r="234" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="D234" s="8"/>
+      <c r="D234" s="7"/>
     </row>
     <row r="235" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
@@ -3390,7 +3412,7 @@
       <c r="C239">
         <v>10000</v>
       </c>
-      <c r="D239" s="8" t="s">
+      <c r="D239" s="7" t="s">
         <v>124</v>
       </c>
     </row>
@@ -3404,7 +3426,7 @@
       <c r="C240">
         <v>0</v>
       </c>
-      <c r="D240" s="8" t="s">
+      <c r="D240" s="7" t="s">
         <v>126</v>
       </c>
     </row>
@@ -3418,7 +3440,7 @@
       <c r="C241">
         <v>0.03</v>
       </c>
-      <c r="D241" s="8" t="s">
+      <c r="D241" s="7" t="s">
         <v>128</v>
       </c>
     </row>
@@ -3432,7 +3454,7 @@
       <c r="C242">
         <v>1</v>
       </c>
-      <c r="D242" s="8" t="s">
+      <c r="D242" s="7" t="s">
         <v>130</v>
       </c>
     </row>
@@ -3446,7 +3468,7 @@
       <c r="C243">
         <v>1</v>
       </c>
-      <c r="D243" s="8" t="s">
+      <c r="D243" s="7" t="s">
         <v>132</v>
       </c>
     </row>
@@ -3456,16 +3478,16 @@
       </c>
     </row>
     <row r="245" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="D245" s="8"/>
+      <c r="D245" s="7"/>
     </row>
     <row r="246" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="D246" s="8"/>
+      <c r="D246" s="7"/>
     </row>
     <row r="247" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A247" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="D247" s="8"/>
+      <c r="D247" s="7"/>
     </row>
     <row r="248" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A248" t="s">
@@ -3474,7 +3496,7 @@
       <c r="B248" t="s">
         <v>2</v>
       </c>
-      <c r="D248" s="8"/>
+      <c r="D248" s="7"/>
     </row>
     <row r="249" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A249" t="s">
@@ -3483,52 +3505,52 @@
       <c r="B249">
         <v>1</v>
       </c>
-      <c r="D249" s="8"/>
+      <c r="D249" s="7"/>
     </row>
     <row r="250" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A250" s="6" t="s">
+      <c r="A250" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="B250" s="6">
+      <c r="B250" s="5">
         <v>3034</v>
       </c>
-      <c r="D250" s="8" t="s">
+      <c r="D250" s="7" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="251" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A251" s="6" t="s">
+      <c r="A251" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="B251" s="6"/>
-      <c r="D251" s="8"/>
+      <c r="B251" s="5"/>
+      <c r="D251" s="7"/>
     </row>
     <row r="252" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A252" t="s">
         <v>127</v>
       </c>
-      <c r="B252" s="6">
+      <c r="B252" s="5">
         <v>0.03</v>
       </c>
-      <c r="D252" s="8"/>
+      <c r="D252" s="7"/>
     </row>
     <row r="253" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A253" t="s">
         <v>165</v>
       </c>
-      <c r="B253" s="6">
+      <c r="B253" s="5">
         <v>50</v>
       </c>
-      <c r="D253" s="8"/>
+      <c r="D253" s="7"/>
     </row>
     <row r="254" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A254" s="6" t="s">
+      <c r="A254" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="B254" s="6">
-        <v>1</v>
-      </c>
-      <c r="D254" s="8" t="s">
+      <c r="B254" s="5">
+        <v>1</v>
+      </c>
+      <c r="D254" s="7" t="s">
         <v>172</v>
       </c>
     </row>

</xml_diff>